<commit_message>
Mise à jour page Lambris
</commit_message>
<xml_diff>
--- a/prix/lambris.xlsx
+++ b/prix/lambris.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\lambris\prix\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\lambris\prix\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{172F69D7-3933-436F-A1F7-69FED6FB9F68}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F023C91-78E5-44C8-9C25-70C6BB20D3B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22932" yWindow="-108" windowWidth="19416" windowHeight="11016" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{6E95DC93-531D-460D-9A06-44397A8920D7}"/>
   </bookViews>
   <sheets>
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="27">
   <si>
     <t>path</t>
   </si>
@@ -102,6 +102,21 @@
   </si>
   <si>
     <t>726158</t>
+  </si>
+  <si>
+    <t>galerie/millim.jpg</t>
+  </si>
+  <si>
+    <t>galerie/cristo.jpg</t>
+  </si>
+  <si>
+    <t>galerie/sarezzi.jpg</t>
+  </si>
+  <si>
+    <t>galerie/blanc-sat.jpg</t>
+  </si>
+  <si>
+    <t>galerie/blanc-brillant.jpg</t>
   </si>
 </sst>
 </file>
@@ -613,7 +628,9 @@
       <c r="G1" s="2"/>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="5"/>
+      <c r="A2" s="5" t="s">
+        <v>22</v>
+      </c>
       <c r="B2" s="21" t="s">
         <v>13</v>
       </c>
@@ -634,7 +651,9 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
+      <c r="A3" s="5" t="s">
+        <v>23</v>
+      </c>
       <c r="B3" s="21" t="s">
         <v>14</v>
       </c>
@@ -655,7 +674,9 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
+      <c r="A4" s="5" t="s">
+        <v>24</v>
+      </c>
       <c r="B4" s="21" t="s">
         <v>15</v>
       </c>
@@ -676,7 +697,9 @@
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
+      <c r="A5" s="5" t="s">
+        <v>25</v>
+      </c>
       <c r="B5" s="21" t="s">
         <v>16</v>
       </c>
@@ -697,7 +720,9 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="5"/>
+      <c r="A6" s="5" t="s">
+        <v>26</v>
+      </c>
       <c r="B6" s="21" t="s">
         <v>17</v>
       </c>

</xml_diff>